<commit_message>
data(gold): sincroniza ES2 com repo reprocessado (+4 materiais)
Repo ES2 foi reprocessado: 25->29 materiais, lessons_index 15->18 datas
(sessoes de julho: Prova P2/PS). Regenerado:
- sarc_subtopics_ES2.csv: 15->17 subtopicos; clean {1-4,6-8,10-17}.
- gold_ES2_rotular.xlsx: 29 materiais, aba subtopico.
- build_ground_truth.py: ES2 clean_subtopics = set(range(1,18))-{5,9}.

Nota: subt 16 (semana Prova P2, 29/06+03/07) agora STRADDLE bloco-11/12
-> precisara de obs se material cair la (ES2 antes era 0-straddle).

MF/SO/TCC verificados identicos ao repo (sem mudanca). IA reprocessado
com renames mas regua 44/6 intacta (renomeados nao sao discriminantes).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRQpbp1NNFwNrJaHsq41XT
</commit_message>
<xml_diff>
--- a/docs/reports/gold_templates/gold_ES2_rotular.xlsx
+++ b/docs/reports/gold_templates/gold_ES2_rotular.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -694,7 +694,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>microsservicos2.pdf</t>
+          <t>Azure.pdf</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>microsservicos2</t>
+          <t>Azure</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>microsservicos3.pdf</t>
+          <t>microsservicos.pdf</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>microsservicos3</t>
+          <t>microsservicos</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>microsservicos5.pdf</t>
+          <t>microsservicos2.pdf</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>microsservicos5</t>
+          <t>microsservicos2</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
@@ -763,7 +763,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>microsservicos6.pdf</t>
+          <t>microsservicos3.pdf</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>microsservicos6</t>
+          <t>microsservicos3</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
@@ -786,7 +786,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>microsservicos7.pdf</t>
+          <t>microsservicos4.pdf</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>microsservicos7</t>
+          <t>microsservicos4</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
@@ -809,7 +809,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>plano.pdf</t>
+          <t>microsservicos5.pdf</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>plano</t>
+          <t>microsservicos5</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
@@ -832,7 +832,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>RevisaoArquiteturaPadroes.pdf</t>
+          <t>microsservicos6.pdf</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Revisao Arquitetura Padroes</t>
+          <t>microsservicos6</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Roteiro1_introducao.pdf</t>
+          <t>microsservicos7.pdf</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Roteiro1 introducao</t>
+          <t>microsservicos7</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
@@ -878,7 +878,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Roteiro2_nameserver.pdf</t>
+          <t>plano.pdf</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Roteiro2 nameserver</t>
+          <t>plano</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Roteiro4_circuitbreaker.pdf</t>
+          <t>RevisaoArquiteturaPadroes.pdf</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Roteiro4 circuitbreaker</t>
+          <t>Revisao Arquitetura Padroes</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
@@ -924,7 +924,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Roteiro5_conteiners.pdf</t>
+          <t>Roteiro1_introducao.pdf</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Roteiro5 conteiners</t>
+          <t>Roteiro1 introducao</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
@@ -947,7 +947,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Roteiro6_conteiners_composicao.pdf</t>
+          <t>Roteiro2_nameserver.pdf</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Roteiro6 conteiners composicao</t>
+          <t>Roteiro2 nameserver</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
@@ -970,7 +970,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Roteiro7_filas.pdf</t>
+          <t>Roteiro3_gateway.pdf</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Roteiro7 filas</t>
+          <t>Roteiro3 gateway</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -993,7 +993,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Roteiro8_autenticacao_autorizacao.pdf</t>
+          <t>Roteiro4_circuitbreaker.pdf</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Roteiro8 autenticacao autorizacao</t>
+          <t>Roteiro4 circuitbreaker</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>servicos.pdf</t>
+          <t>Roteiro5_conteiners.pdf</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>Roteiro5 conteiners</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>t1_2026_1.pdf</t>
+          <t>Roteiro6_conteiners_composicao.pdf</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>t1 2026 1</t>
+          <t>Roteiro6 conteiners composicao</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>web.pdf</t>
+          <t>Roteiro7_filas.pdf</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1072,20 +1072,112 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>Roteiro7 filas</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
       <c r="F26" s="5" t="inlineStr"/>
       <c r="G26" s="6" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Roteiro8_autenticacao_autorizacao.pdf</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Roteiro8 autenticacao autorizacao</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>servicos.pdf</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>t1_2026_1.pdf</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>t1 2026 1</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>web.pdf</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
   <dataValidations count="2">
-    <dataValidation sqref="E2:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Escolha um subtópico da lista (ou N/A / não sei)." prompt="Selecione o subtópico correto (SARC)." type="list">
-      <formula1>'Gabarito Subtopicos'!$F$2:$F$16</formula1>
+    <dataValidation sqref="E2:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Escolha um subtópico da lista (ou N/A / não sei)." prompt="Selecione o subtópico correto (SARC)." type="list">
+      <formula1>'Gabarito Subtopicos'!$F$2:$F$18</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="Sua confiança na resposta." type="list">
+    <dataValidation sqref="F2:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="Sua confiança na resposta." type="list">
       <formula1>"alta,média,baixa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1099,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1528,7 +1620,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>15 — implantação de microsserviços em conteiners</t>
+          <t>15 — DevOps</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1650,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>16 — implantação de microsserviços em conteiners / Prova P2, Entrega trabalho</t>
         </is>
       </c>
     </row>
@@ -1568,25 +1660,81 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>implantação de microsserviços em conteiners</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>29/06</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
+          <t>26/06</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Roteiro (Moodle)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>17 — Prova PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>implantação de microsserviços em conteiners / Prova P2, Entrega trabalho</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>29/06, 03/07</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Deploy/Conteiners</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Roteiro (Moodle)</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Prova PS</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Avaliação</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Roteiro (Moodle)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>não sei</t>
         </is>

</xml_diff>